<commit_message>
Team carousel: 8 people, human traits instead of job titles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmVGpe1UCrVUCKrYMjR91a
</commit_message>
<xml_diff>
--- a/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
+++ b/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Carrossel: Conheça quem cuida (time completo)</t>
+          <t>Carrossel: Conheça quem cuida (time completo, sem cargos)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -904,27 +904,30 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Quem cuida de quem cuida da sua empresa.</t>
+          <t>Quem cuida. (sub: 8 pessoas, uma mesma pergunta)</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>1 · CAPA · Foto do time junto. Título: Quem cuida de quem cuida da sua empresa.
-2 · Somos médicos, psicólogos e profissionais de saúde que acreditam em uma coisa: cuidado começa pela pessoa.
-3 · Dr. Ronald · [função na FAIR HEALTH] · "O que importa para você?" → [resposta dele, 1 frase]
-4 · Dra. Floriana · [função] · "O que importa para você?" → [resposta]
-5 · Dra. Marília · [função] · "O que importa para você?" → [resposta]
-6 · Nina · [função] · "O que importa para você?" → [resposta]
-7 · [Integrante #5] · [função] · "O que importa para você?" → [resposta]
-8 · Diferentes formações, a mesma pergunta no começo de todo cuidado.
-9 · CTA · E para você, o que importa? Conta aqui nos comentários.</t>
+          <t>MODELO DE SLIDE DE PESSOA: foto grande · frase humana em destaque · "O que importa para você?" + resposta da pessoa (1 frase) · nome pequeno no rodapé. Sem cargo.
+1 · CAPA · Foto do time junto. "Quem cuida." / Sub: 8 pessoas, uma mesma pergunta.
+2 · Antes de cuidar de alguém, a gente pergunta: o que importa para você? Fizemos essa pergunta a nós mesmos.
+3 · Marília · "Acredita que arte e cura andam juntas. Atriz e cantora nas horas vagas." · O que importa: [resposta]
+4 · Nina · "Escreve código e estuda Nutrição, para a tecnologia falar a língua do cuidado." · O que importa: [resposta]
+5 · Ronald · [RASCUNHO] "Passou a vida cuidando de crianças, adolescentes e atletas." · O que importa: [resposta]
+6 · Floriana · [RASCUNHO] "Professora e autora: gosta de transformar ciência em conversa." · O que importa: [resposta]
+7 · Renata · [RASCUNHO] "Entre a sala de aula e a psicologia, aprendeu que ouvir muda o trabalho." · O que importa: [resposta]
+8 · Liliane · [RASCUNHO] "Acredita que qualidade de vida se constrói no dia a dia, não só nas férias." · O que importa: [resposta]
+9 · Fernando · [RASCUNHO] "Curioso sobre o cérebro humano e sobre como as pessoas trabalham melhor." · O que importa: [resposta]
+10 · Charles · [RASCUNHO] "Sempre começa perguntando como é estar do outro lado." · O que importa: [resposta]
+11 · CTA · Diferentes histórias, a mesma pergunta no começo de todo cuidado. E para você, o que importa? Conta nos comentários.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Por trás de todo cuidado, tem gente.
-Estas são as pessoas que fazem a FAIR HEALTH acontecer: médicos, psicólogos e profissionais que escolheram cuidar antes que o adoecimento vire afastamento.
-Perguntamos a cada um a mesma coisa que perguntamos a quem atendemos: o que importa para você? As respostas estão no carrossel.
+Antes de cuidar de alguém, a gente pergunta o que importa para aquela pessoa. Então decidimos começar por nós mesmos.
+São 8 pessoas com histórias bem diferentes: tem quem cante, quem escreva código, quem passe o dia em sala de aula. Todo mundo respondeu à mesma pergunta, e as respostas estão no carrossel.
 E para você, o que importa?
 #fairhealth #saudecorporativa #cuidadocentradonapessoa #medicinadoestilodevida #saudedotrabalhador</t>
         </is>
@@ -941,7 +944,7 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>Retrato individual de cada um (cena C1) + foto do time junto (C2)</t>
+          <t>8 pessoas: Marília, Nina, Ronald, Floriana, Renata, Liliane, Fernando, Charles. Retrato de cada um (C1) + foto do time (C2)</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -951,7 +954,7 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>Mesmo modelo visual para todos os slides de pessoa. Pendente: nome do integrante #5, funções e respostas.</t>
+          <t>Pedido do sócio: sem cargo, destacar características humanas. Frases de Marília e Nina vêm do slide do time; as marcadas RASCUNHO precisam ser validadas por cada pessoa (questionário de 3 perguntas). Confirmar com o Dr. Ronald se os médicos precisam de CRM no post (regra de publicidade médica).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Team carousel as placeholder structure for approval
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmVGpe1UCrVUCKrYMjR91a
</commit_message>
<xml_diff>
--- a/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
+++ b/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
@@ -909,17 +909,17 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>MODELO DE SLIDE DE PESSOA: foto grande · frase humana em destaque · "O que importa para você?" + resposta da pessoa (1 frase) · nome pequeno no rodapé. Sem cargo.
+          <t>MODELO DE SLIDE DE PESSOA: [FOTO] grande · [FRASE HUMANA] em destaque · "O que importa para você?" + [RESPOSTA] · nome no rodapé. Sem cargo. Fotos e textos serão pedidos na aprovação.
 1 · CAPA · Foto do time junto. "Quem cuida." / Sub: 8 pessoas, uma mesma pergunta.
 2 · Antes de cuidar de alguém, a gente pergunta: o que importa para você? Fizemos essa pergunta a nós mesmos.
-3 · Marília · "Acredita que arte e cura andam juntas. Atriz e cantora nas horas vagas." · O que importa: [resposta]
-4 · Nina · "Escreve código e estuda Nutrição, para a tecnologia falar a língua do cuidado." · O que importa: [resposta]
-5 · Ronald · [RASCUNHO] "Passou a vida cuidando de crianças, adolescentes e atletas." · O que importa: [resposta]
-6 · Floriana · [RASCUNHO] "Professora e autora: gosta de transformar ciência em conversa." · O que importa: [resposta]
-7 · Renata · [RASCUNHO] "Entre a sala de aula e a psicologia, aprendeu que ouvir muda o trabalho." · O que importa: [resposta]
-8 · Liliane · [RASCUNHO] "Acredita que qualidade de vida se constrói no dia a dia, não só nas férias." · O que importa: [resposta]
-9 · Fernando · [RASCUNHO] "Curioso sobre o cérebro humano e sobre como as pessoas trabalham melhor." · O que importa: [resposta]
-10 · Charles · [RASCUNHO] "Sempre começa perguntando como é estar do outro lado." · O que importa: [resposta]
+3 · Marília · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
+4 · Nina · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
+5 · Ronald · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
+6 · Floriana · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
+7 · Renata · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
+8 · Liliane · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
+9 · Fernando · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
+10 · Charles · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
 11 · CTA · Diferentes histórias, a mesma pergunta no começo de todo cuidado. E para você, o que importa? Conta nos comentários.</t>
         </is>
       </c>
@@ -927,7 +927,7 @@
         <is>
           <t>Por trás de todo cuidado, tem gente.
 Antes de cuidar de alguém, a gente pergunta o que importa para aquela pessoa. Então decidimos começar por nós mesmos.
-São 8 pessoas com histórias bem diferentes: tem quem cante, quem escreva código, quem passe o dia em sala de aula. Todo mundo respondeu à mesma pergunta, e as respostas estão no carrossel.
+São 8 pessoas com histórias bem diferentes. Todo mundo respondeu à mesma pergunta, e as respostas estão no carrossel.
 E para você, o que importa?
 #fairhealth #saudecorporativa #cuidadocentradonapessoa #medicinadoestilodevida #saudedotrabalhador</t>
         </is>
@@ -949,12 +949,12 @@
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Em revisão</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>Pedido do sócio: sem cargo, destacar características humanas. Frases de Marília e Nina vêm do slide do time; as marcadas RASCUNHO precisam ser validadas por cada pessoa (questionário de 3 perguntas). Confirmar com o Dr. Ronald se os médicos precisam de CRM no post (regra de publicidade médica).</t>
+          <t>Estrutura para aprovação: fotos, frases e respostas serão pedidas a cada pessoa na aprovação. Sem cargo (pedido do sócio). Confirmar com o Dr. Ronald se os médicos precisam de CRM no post.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Team carousel: elegant title-only cover, 'Cuidar, para mim, é…' prompt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmVGpe1UCrVUCKrYMjR91a
</commit_message>
<xml_diff>
--- a/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
+++ b/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Carrossel: Conheça quem cuida (time completo, sem cargos)</t>
+          <t>Carrossel: Quem cuida (time completo, sem cargos)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -904,37 +904,37 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Quem cuida. (sub: 8 pessoas, uma mesma pergunta)</t>
+          <t>Quem cuida. (capa só com título grande e flecha; sem foto)</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>MODELO DE SLIDE DE PESSOA: [FOTO] grande · [FRASE HUMANA] em destaque · "O que importa para você?" + [RESPOSTA] · nome no rodapé. Sem cargo. Fotos e textos serão pedidos na aprovação.
-1 · CAPA · Foto do time junto. "Quem cuida." / Sub: 8 pessoas, uma mesma pergunta.
-2 · Antes de cuidar de alguém, a gente pergunta: o que importa para você? Fizemos essa pergunta a nós mesmos.
-3 · Marília · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-4 · Nina · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-5 · Ronald · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-6 · Floriana · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-7 · Renata · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-8 · Liliane · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-9 · Fernando · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-10 · Charles · [FOTO] · [FRASE HUMANA] · O que importa para você? → [RESPOSTA]
-11 · CTA · Diferentes histórias, a mesma pergunta no começo de todo cuidado. E para você, o que importa? Conta nos comentários.</t>
+          <t>MODELO DE SLIDE DE PESSOA: [FOTO] · nome · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]. Sem cargo.
+1 · CAPA · Fundo verde-escuro. Pequeno no topo: O TIME FAIR HEALTH. Título grande: Quem cuida. Sub: 8 pessoas por trás de cada cuidado. Flecha para o lado.
+2 · Por trás de cada cuidado, tem gente. Pedimos a cada pessoa do time que completasse uma frase: "Cuidar, para mim, é…"
+3 · Marília · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+4 · Nina · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+5 · Ronald · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+6 · Floriana · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+7 · Renata · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+8 · Liliane · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+9 · Fernando · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+10 · Charles · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
+11 · CTA · Histórias diferentes, o mesmo jeito de cuidar. E para você, o que é cuidar? Conta nos comentários.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Por trás de todo cuidado, tem gente.
-Antes de cuidar de alguém, a gente pergunta o que importa para aquela pessoa. Então decidimos começar por nós mesmos.
-São 8 pessoas com histórias bem diferentes. Todo mundo respondeu à mesma pergunta, e as respostas estão no carrossel.
-E para você, o que importa?
+Pedimos a cada pessoa do time da FAIR HEALTH que completasse uma frase: "Cuidar, para mim, é…". As respostas estão no carrossel.
+São 8 histórias diferentes e um mesmo jeito de cuidar: começando pela pessoa.
+E para você, o que é cuidar?
 #fairhealth #saudecorporativa #cuidadocentradonapessoa #medicinadoestilodevida #saudedotrabalhador</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Comente: e para você, o que importa?</t>
+          <t>Comente: e para você, o que é cuidar?</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>8 pessoas: Marília, Nina, Ronald, Floriana, Renata, Liliane, Fernando, Charles. Retrato de cada um (C1) + foto do time (C2)</t>
+          <t>8 pessoas: Marília, Nina, Ronald, Floriana, Renata, Liliane, Fernando, Charles. Retrato individual de cada um.</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>Estrutura para aprovação: fotos, frases e respostas serão pedidas a cada pessoa na aprovação. Sem cargo (pedido do sócio). Confirmar com o Dr. Ronald se os médicos precisam de CRM no post.</t>
+          <t>Na aprovação, pedir a cada pessoa: 1) uma foto (fundo claro, do peito para cima); 2) completar "Cuidar, para mim, é…"; 3) o que gosta de fazer fora do trabalho. Sem cargo (pedido do sócio). Confirmar com o Dr. Ronald se médicos precisam de CRM no post. Arte: instagram/posts/time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Team carousel in editorial style (serif names, full-bleed portraits, 'Ama' line)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmVGpe1UCrVUCKrYMjR91a
</commit_message>
<xml_diff>
--- a/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
+++ b/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Carrossel: Quem cuida (time completo, sem cargos)</t>
+          <t>Carrossel: Nosso Time (8 pessoas, sem cargos)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -904,30 +904,29 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Quem cuida. (capa só com título grande e flecha; sem foto)</t>
+          <t>Nosso Time. (sub: Conheça quem cuida da saúde da sua empresa.)</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>MODELO DE SLIDE DE PESSOA: [FOTO] · nome · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]. Sem cargo.
-1 · CAPA · Fundo verde-escuro. Pequeno no topo: O TIME FAIR HEALTH. Título grande: Quem cuida. Sub: 8 pessoas por trás de cada cuidado. Flecha para o lado.
-2 · Por trás de cada cuidado, tem gente. Pedimos a cada pessoa do time que completasse uma frase: "Cuidar, para mim, é…"
-3 · Marília · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-4 · Nina · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-5 · Ronald · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-6 · Floriana · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-7 · Renata · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-8 · Liliane · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-9 · Fernando · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-10 · Charles · [FOTO] · "Cuidar, para mim, é [resposta]." · Fora daqui: [o que gosta de fazer]
-11 · CTA · Histórias diferentes, o mesmo jeito de cuidar. E para você, o que é cuidar? Conta nos comentários.</t>
+          <t>ESTILO: editorial (referência @conselhosdorh): título em serifa, retrato em tela cheia, bloco pequeno com linha vertical verde-água. Sem cargo.
+1 · CAPA · Fundo claro, sem foto. "Nosso Time" grande em serifa (Time em itálico verde). Sub: Conheça quem cuida da saúde da sua empresa. Flecha para o lado.
+2 · Marília · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+3 · Nina · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+4 · Ronald · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+5 · Floriana · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+6 · Renata · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+7 · Liliane · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+8 · Fernando · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+9 · Charles · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
+10 · FECHAMENTO · Fundo verde-escuro: Pessoas diferentes, um mesmo jeito de cuidar. E para você, o que é cuidar? Conta nos comentários. Logo.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Por trás de todo cuidado, tem gente.
-Pedimos a cada pessoa do time da FAIR HEALTH que completasse uma frase: "Cuidar, para mim, é…". As respostas estão no carrossel.
-São 8 histórias diferentes e um mesmo jeito de cuidar: começando pela pessoa.
+Estas são as pessoas que fazem a FAIR HEALTH acontecer. Cada uma com a sua história, as suas paixões e o seu jeito de explicar o que é cuidar.
+O que une todo mundo é o ponto de partida: antes de qualquer plano, a gente pergunta o que importa para você.
 E para você, o que é cuidar?
 #fairhealth #saudecorporativa #cuidadocentradonapessoa #medicinadoestilodevida #saudedotrabalhador</t>
         </is>
@@ -944,7 +943,7 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>8 pessoas: Marília, Nina, Ronald, Floriana, Renata, Liliane, Fernando, Charles. Retrato individual de cada um.</t>
+          <t>8 pessoas: Marília, Nina, Ronald, Floriana, Renata, Liliane, Fernando, Charles. Retrato individual, vertical, luz natural, fundo real.</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -954,7 +953,7 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>Na aprovação, pedir a cada pessoa: 1) uma foto (fundo claro, do peito para cima); 2) completar "Cuidar, para mim, é…"; 3) o que gosta de fazer fora do trabalho. Sem cargo (pedido do sócio). Confirmar com o Dr. Ronald se médicos precisam de CRM no post. Arte: instagram/posts/time.</t>
+          <t>Na aprovação, pedir a cada pessoa: 1) retrato vertical (luz natural, fundo real, sorrindo); 2) complete "Cuidar é…" em poucas palavras; 3) três coisas que ama (ex.: Treinar | Viajar | Família). Sem cargo (pedido do sócio). Confirmar CRM dos médicos com o Dr. Ronald. Arte: instagram/posts/time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Team carousel back to brand fonts/colors; reference composition only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmVGpe1UCrVUCKrYMjR91a
</commit_message>
<xml_diff>
--- a/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
+++ b/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Carrossel: Nosso Time (8 pessoas, sem cargos)</t>
+          <t>Carrossel: Nosso time (8 pessoas, sem cargos)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -904,36 +904,36 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Nosso Time. (sub: Conheça quem cuida da saúde da sua empresa.)</t>
+          <t>Nosso time. (sub: Conheça quem cuida da saúde da sua empresa.)</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>ESTILO: editorial (referência @conselhosdorh): título em serifa, retrato em tela cheia, bloco pequeno com linha vertical verde-água. Sem cargo.
-1 · CAPA · Fundo claro, sem foto. "Nosso Time" grande em serifa (Time em itálico verde). Sub: Conheça quem cuida da saúde da sua empresa. Flecha para o lado.
-2 · Marília · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-3 · Nina · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-4 · Ronald · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-5 · Floriana · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-6 · Renata · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-7 · Liliane · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-8 · Fernando · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-9 · Charles · [FOTO em tela cheia] · nome grande em serifa no topo · "Cuidar é [resposta curta]." · Ama: [ ] | [ ] | [ ]
-10 · FECHAMENTO · Fundo verde-escuro: Pessoas diferentes, um mesmo jeito de cuidar. E para você, o que é cuidar? Conta nos comentários. Logo.</t>
+          <t>IDENTIDADE: fontes e cores da marca (Raleway, verde-escuro, verde-água). Da referência @conselhosdorh só a composição: retrato em tela cheia, nome no topo, bloco com linha vertical embaixo. Sem cargo.
+1 · CAPA · Verde-escuro, sem foto. FAIR HEALTH pequeno no topo. "Nosso time." grande. Sub: Conheça quem cuida da saúde da sua empresa. Flecha para o lado.
+2 · Marília · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+3 · Nina · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+4 · Ronald · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+5 · Floriana · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+6 · Renata · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+7 · Liliane · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+8 · Fernando · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+9 · Charles · [FOTO em tela cheia] · nome grande no topo · bloco com linha verde-água: [pequena descrição] / O que é importante para você? [resposta]
+10 · FECHAMENTO · Verde-escuro: Pessoas diferentes, um mesmo jeito de cuidar. E para você, o que é importante? Conta nos comentários. Logo.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Por trás de todo cuidado, tem gente.
-Estas são as pessoas que fazem a FAIR HEALTH acontecer. Cada uma com a sua história, as suas paixões e o seu jeito de explicar o que é cuidar.
-O que une todo mundo é o ponto de partida: antes de qualquer plano, a gente pergunta o que importa para você.
-E para você, o que é cuidar?
+Estas são as pessoas que fazem a FAIR HEALTH acontecer, cada uma com a sua história.
+Fizemos a todas a mesma pergunta que fazemos a quem cuidamos: o que é importante para você? As respostas estão no carrossel.
+E para você, o que é importante?
 #fairhealth #saudecorporativa #cuidadocentradonapessoa #medicinadoestilodevida #saudedotrabalhador</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Comente: e para você, o que é cuidar?</t>
+          <t>Comente: e para você, o que é importante?</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>8 pessoas: Marília, Nina, Ronald, Floriana, Renata, Liliane, Fernando, Charles. Retrato individual, vertical, luz natural, fundo real.</t>
+          <t>8 pessoas: Marília, Nina, Ronald, Floriana, Renata, Liliane, Fernando, Charles. Retrato individual vertical.</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>Na aprovação, pedir a cada pessoa: 1) retrato vertical (luz natural, fundo real, sorrindo); 2) complete "Cuidar é…" em poucas palavras; 3) três coisas que ama (ex.: Treinar | Viajar | Família). Sem cargo (pedido do sócio). Confirmar CRM dos médicos com o Dr. Ronald. Arte: instagram/posts/time.</t>
+          <t>Na aprovação, pedir a cada pessoa: 1) retrato vertical (luz natural, fundo real); 2) uma pequena descrição sobre si, sem cargo; 3) resposta curta a "O que é importante para você?". Confirmar CRM dos médicos com o Dr. Ronald. Arte: instagram/posts/time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add brand presentation carousel (post 2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmVGpe1UCrVUCKrYMjR91a
</commit_message>
<xml_diff>
--- a/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
+++ b/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
@@ -814,12 +814,12 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>1 · CAPA · O afastamento não começa no atestado. / Bem-vindos à FAIR HEALTH.
+          <t>1 · CAPA · Verde-escuro. BEM-VINDOS À FAIR HEALTH pequeno no topo. O afastamento não começa no atestado. / Por que a FAIR HEALTH existe. Flecha.
 2 · Quando vira atestado, o adoecimento já começou faz tempo.
 3 · O RH costuma enxergar só o fim da história: atestado, afastamento e sinistro no plano de saúde.
 4 · E o começo é pequeno: sono ruim, estresse acumulado, um hábito que escorrega, uma dor que ninguém trata.
 5 · Por isso levamos o cuidado para dentro da empresa: médicos, psicólogos e assistentes sociais onde o time já está.
-6 · E começamos com uma pergunta: O que importa para você? Rotina, objetivos e contexto viram um plano de cuidado individual, baseado na Medicina do Estilo de Vida.
+6 · E todo cuidado começa com uma pergunta: O que importa para você? Rotina, objetivos e contexto viram um plano de cuidado individual, baseado na Medicina do Estilo de Vida.
 7 · E comprovamos com dados: o RH recebe relatórios anonimizados. Nenhum dado individual.
 8 · RESUMO · Por que existimos: 1. O adoecimento começa antes do atestado. 2. O RH só vê o fim. 3. Cuidado precisa estar perto. 4. Cada pessoa tem um plano. 5. Comprovamos com dados.
 9 · CTA · Siga @fairhealth.br e conheça quem cuida.</t>
@@ -852,12 +852,12 @@
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>Em produção</t>
+          <t>Em revisão</t>
         </is>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>Base: arte já pronta em instagram/posts/estreia (carrossel #1). Incluir o slide 6 novo.</t>
+          <t>Arte pronta: instagram/posts/marca (9 slides, mesma capa do carrossel do time). Pronto para aprovação.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add November 2026 calendar (1 to 30) to the content schedule
New 'Novembro' sheet with every day of the month, reusing the November
posts from the 90-day plan and pulling proof and conversion forward
(Chemitec, HDSA, testimonials, NR-01 guide, free diagnosis) into the HR
budget window. Holidays without posts, polls moved to Stories, Novembro
Azul added. Includes dependencies and what moves to December, plus a
'Novembro (calendário)' month grid for sharing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CtZHU3TZMahhA8PyMk16cb
</commit_message>
<xml_diff>
--- a/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
+++ b/marketing/Cronograma_Conteudo_FairHealth_90dias.xlsx
@@ -8,10 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Novembro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Novembro (calendário)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cronograma'!$A$4:$Q$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Novembro'!$A$4:$Q$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,11 +23,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="dd/mm (ddd)"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm (ddd)"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +68,30 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005F6B69"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002F6B64"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00141B1B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00141B1B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -88,8 +113,33 @@
         <fgColor rgb="00F4F8F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF1F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF6E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F2EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6F8F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -111,15 +161,29 @@
         <color rgb="00C9D6D3"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D3D1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9D3D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D3D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D3D1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -130,7 +194,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -142,17 +206,65 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -178,6 +290,38 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFF3C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6E8D5"/>
+          <bgColor rgb="00C6E8D5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E3F1DC"/>
+          <bgColor rgb="00E3F1DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE8C8"/>
+          <bgColor rgb="00FCE8C8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF3C4"/>
+          <bgColor rgb="00FFF3C4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -578,7 +722,7 @@
           <t>Início (segunda da semana 1):</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="14" t="n">
         <v>46300</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -686,7 +830,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="15">
         <f>$D$2+(B5-1)*7+MATCH(C5,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -778,7 +922,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="15">
         <f>$D$2+(B6-1)*7+MATCH(C6,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -873,7 +1017,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="15">
         <f>$D$2+(B7-1)*7+MATCH(C7,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -969,7 +1113,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="15">
         <f>$D$2+(B8-1)*7+MATCH(C8,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1023,7 +1167,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="15">
         <f>$D$2+(B9-1)*7+MATCH(C9,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1081,7 +1225,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="16">
         <f>$D$2+(B10-1)*7+MATCH(C10,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1135,7 +1279,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="16">
         <f>$D$2+(B11-1)*7+MATCH(C11,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1189,7 +1333,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="16">
         <f>$D$2+(B12-1)*7+MATCH(C12,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1243,7 +1387,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="16">
         <f>$D$2+(B13-1)*7+MATCH(C13,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1297,7 +1441,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="16">
         <f>$D$2+(B14-1)*7+MATCH(C14,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1351,7 +1495,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="15">
         <f>$D$2+(B15-1)*7+MATCH(C15,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1405,7 +1549,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="15">
         <f>$D$2+(B16-1)*7+MATCH(C16,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1459,7 +1603,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="15">
         <f>$D$2+(B17-1)*7+MATCH(C17,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1513,7 +1657,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="15">
         <f>$D$2+(B18-1)*7+MATCH(C18,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1567,7 +1711,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="15">
         <f>$D$2+(B19-1)*7+MATCH(C19,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1621,7 +1765,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="16">
         <f>$D$2+(B20-1)*7+MATCH(C20,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1675,7 +1819,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="16">
         <f>$D$2+(B21-1)*7+MATCH(C21,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1729,7 +1873,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="16">
         <f>$D$2+(B22-1)*7+MATCH(C22,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1783,7 +1927,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="16">
         <f>$D$2+(B23-1)*7+MATCH(C23,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1837,7 +1981,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="16">
         <f>$D$2+(B24-1)*7+MATCH(C24,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1891,7 +2035,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D25" s="8">
+      <c r="D25" s="15">
         <f>$D$2+(B25-1)*7+MATCH(C25,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1945,7 +2089,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D26" s="8">
+      <c r="D26" s="15">
         <f>$D$2+(B26-1)*7+MATCH(C26,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -1999,7 +2143,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="15">
         <f>$D$2+(B27-1)*7+MATCH(C27,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2053,7 +2197,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D28" s="8">
+      <c r="D28" s="15">
         <f>$D$2+(B28-1)*7+MATCH(C28,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2107,7 +2251,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="15">
         <f>$D$2+(B29-1)*7+MATCH(C29,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2161,7 +2305,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="16">
         <f>$D$2+(B30-1)*7+MATCH(C30,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2215,7 +2359,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="16">
         <f>$D$2+(B31-1)*7+MATCH(C31,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2269,7 +2413,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="16">
         <f>$D$2+(B32-1)*7+MATCH(C32,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2323,7 +2467,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="16">
         <f>$D$2+(B33-1)*7+MATCH(C33,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2377,7 +2521,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="16">
         <f>$D$2+(B34-1)*7+MATCH(C34,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2431,7 +2575,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D35" s="8">
+      <c r="D35" s="15">
         <f>$D$2+(B35-1)*7+MATCH(C35,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2485,7 +2629,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D36" s="8">
+      <c r="D36" s="15">
         <f>$D$2+(B36-1)*7+MATCH(C36,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2539,7 +2683,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D37" s="8">
+      <c r="D37" s="15">
         <f>$D$2+(B37-1)*7+MATCH(C37,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2593,7 +2737,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="15">
         <f>$D$2+(B38-1)*7+MATCH(C38,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2647,7 +2791,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D39" s="8">
+      <c r="D39" s="15">
         <f>$D$2+(B39-1)*7+MATCH(C39,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2701,7 +2845,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="16">
         <f>$D$2+(B40-1)*7+MATCH(C40,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2755,7 +2899,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="16">
         <f>$D$2+(B41-1)*7+MATCH(C41,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2809,7 +2953,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="16">
         <f>$D$2+(B42-1)*7+MATCH(C42,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2863,7 +3007,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="16">
         <f>$D$2+(B43-1)*7+MATCH(C43,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2917,7 +3061,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D44" s="12">
+      <c r="D44" s="16">
         <f>$D$2+(B44-1)*7+MATCH(C44,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -2971,7 +3115,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D45" s="8">
+      <c r="D45" s="15">
         <f>$D$2+(B45-1)*7+MATCH(C45,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3025,7 +3169,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D46" s="8">
+      <c r="D46" s="15">
         <f>$D$2+(B46-1)*7+MATCH(C46,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3079,7 +3223,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D47" s="8">
+      <c r="D47" s="15">
         <f>$D$2+(B47-1)*7+MATCH(C47,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3133,7 +3277,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D48" s="8">
+      <c r="D48" s="15">
         <f>$D$2+(B48-1)*7+MATCH(C48,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3187,7 +3331,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D49" s="8">
+      <c r="D49" s="15">
         <f>$D$2+(B49-1)*7+MATCH(C49,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3241,7 +3385,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="16">
         <f>$D$2+(B50-1)*7+MATCH(C50,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3295,7 +3439,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D51" s="12">
+      <c r="D51" s="16">
         <f>$D$2+(B51-1)*7+MATCH(C51,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3349,7 +3493,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D52" s="12">
+      <c r="D52" s="16">
         <f>$D$2+(B52-1)*7+MATCH(C52,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3403,7 +3547,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D53" s="12">
+      <c r="D53" s="16">
         <f>$D$2+(B53-1)*7+MATCH(C53,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3457,7 +3601,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="16">
         <f>$D$2+(B54-1)*7+MATCH(C54,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3511,7 +3655,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D55" s="8">
+      <c r="D55" s="15">
         <f>$D$2+(B55-1)*7+MATCH(C55,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3565,7 +3709,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D56" s="8">
+      <c r="D56" s="15">
         <f>$D$2+(B56-1)*7+MATCH(C56,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3619,7 +3763,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D57" s="8">
+      <c r="D57" s="15">
         <f>$D$2+(B57-1)*7+MATCH(C57,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3673,7 +3817,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D58" s="8">
+      <c r="D58" s="15">
         <f>$D$2+(B58-1)*7+MATCH(C58,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3727,7 +3871,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D59" s="8">
+      <c r="D59" s="15">
         <f>$D$2+(B59-1)*7+MATCH(C59,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3781,7 +3925,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="16">
         <f>$D$2+(B60-1)*7+MATCH(C60,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3835,7 +3979,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="16">
         <f>$D$2+(B61-1)*7+MATCH(C61,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3889,7 +4033,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="16">
         <f>$D$2+(B62-1)*7+MATCH(C62,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3943,7 +4087,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D63" s="12">
+      <c r="D63" s="16">
         <f>$D$2+(B63-1)*7+MATCH(C63,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -3997,7 +4141,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D64" s="12">
+      <c r="D64" s="16">
         <f>$D$2+(B64-1)*7+MATCH(C64,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -4051,7 +4195,7 @@
           <t>Segunda</t>
         </is>
       </c>
-      <c r="D65" s="8">
+      <c r="D65" s="15">
         <f>$D$2+(B65-1)*7+MATCH(C65,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -4105,7 +4249,7 @@
           <t>Terça</t>
         </is>
       </c>
-      <c r="D66" s="8">
+      <c r="D66" s="15">
         <f>$D$2+(B66-1)*7+MATCH(C66,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -4159,7 +4303,7 @@
           <t>Quarta</t>
         </is>
       </c>
-      <c r="D67" s="8">
+      <c r="D67" s="15">
         <f>$D$2+(B67-1)*7+MATCH(C67,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -4213,7 +4357,7 @@
           <t>Quinta</t>
         </is>
       </c>
-      <c r="D68" s="8">
+      <c r="D68" s="15">
         <f>$D$2+(B68-1)*7+MATCH(C68,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -4267,7 +4411,7 @@
           <t>Sexta</t>
         </is>
       </c>
-      <c r="D69" s="8">
+      <c r="D69" s="15">
         <f>$D$2+(B69-1)*7+MATCH(C69,Listas!$A$1:$A$5,0)-1</f>
         <v/>
       </c>
@@ -4343,6 +4487,2968 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002F6B64"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="44" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Calendário de novembro 2026 · FAIR HEALTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Tema do mês: da intenção à evidência. Outubro mostrou quem somos e como cuidamos; novembro prova que funciona e abre a conversa com o RH (janela de orçamento 2027). Ritmo: até 5 posts por semana às 7:30, com 2 Reels por semana; feriados sem post.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Dia</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Tema da semana</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Origem (90 dias)</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Pauta</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Especificação</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Gancho (capa ou 2 s iniciais)</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Roteiro / conteúdo</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Legenda</t>
+        </is>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>CTA</t>
+        </is>
+      </c>
+      <c r="N4" s="18" t="inlineStr">
+        <is>
+          <t>Hashtags</t>
+        </is>
+      </c>
+      <c r="O4" s="18" t="inlineStr">
+        <is>
+          <t>Quem aparece / fotos</t>
+        </is>
+      </c>
+      <c r="P4" s="18" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="Q4" s="18" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="19" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Abertura do mês</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>Stories: Novembro Azul começa hoje</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Abrir o mês e anunciar o tema</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Stories</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · sequência de 3 a 5 telas com figurinha</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>Novembro é mês de falar de saúde do homem.</t>
+        </is>
+      </c>
+      <c r="K5" s="20" t="n"/>
+      <c r="L5" s="20" t="n"/>
+      <c r="M5" s="20" t="inlineStr">
+        <is>
+          <t>Figurinha de pergunta: "O que te faz adiar uma consulta?"</t>
+        </is>
+      </c>
+      <c r="N5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O5" s="20" t="inlineStr">
+        <is>
+          <t>Arte (logo coração)</t>
+        </is>
+      </c>
+      <c r="P5" s="20" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q5" s="20" t="inlineStr">
+        <is>
+          <t>Agendar na sexta 30/10. As respostas da caixa alimentam o Reel de 03/11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="19" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>Feriado: Finados</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>Sem publicação</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" s="20" t="n"/>
+      <c r="L6" s="20" t="n"/>
+      <c r="M6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q6" s="20" t="inlineStr">
+        <is>
+          <t>Feriado nacional. Público de RH fora do ar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="A7" s="21" t="n">
+        <v>46329</v>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Novembro Azul e movimento</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>NOVO</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>1 Minuto de Cuidado: por que o homem só vai ao médico quando dói</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Descoberta, educação e retenção</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="inlineStr">
+        <is>
+          <t>Ele só vai ao médico quando dói.</t>
+        </is>
+      </c>
+      <c r="K7" s="22" t="n"/>
+      <c r="L7" s="22" t="n"/>
+      <c r="M7" s="22" t="inlineStr">
+        <is>
+          <t>Mande para alguém que está adiando a consulta</t>
+        </is>
+      </c>
+      <c r="N7" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #novembroazul #saudedohomem #saudecorporativa #prevencao</t>
+        </is>
+      </c>
+      <c r="O7" s="22" t="inlineStr">
+        <is>
+          <t>Dr. Ronald para a câmera</t>
+        </is>
+      </c>
+      <c r="P7" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q7" s="22" t="inlineStr">
+        <is>
+          <t>Abre a campanha. Sem números sem fonte e sem falar de exame específico como promessa. Revisão técnica do Dr. Ronald. Stories do dia: enquete de movimento (era o ID 21).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1">
+      <c r="A8" s="21" t="n">
+        <v>46330</v>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Quarta</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Novembro Azul e movimento</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>ID 23</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Pilar 2: Atividade física</t>
+        </is>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Autoridade, salvamento e compartilhamento</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J8" s="22" t="inlineStr">
+        <is>
+          <t>Movimento não precisa caber na academia.</t>
+        </is>
+      </c>
+      <c r="K8" s="22" t="n"/>
+      <c r="L8" s="22" t="n"/>
+      <c r="M8" s="22" t="inlineStr">
+        <is>
+          <t>Salve para lembrar na próxima pausa</t>
+        </is>
+      </c>
+      <c r="N8" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O8" s="22" t="inlineStr">
+        <is>
+          <t>Arte estilo pilares (duotone, cor do pilar)</t>
+        </is>
+      </c>
+      <c r="P8" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q8" s="22" t="inlineStr">
+        <is>
+          <t>Série 7 pilares.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="A9" s="21" t="n">
+        <v>46331</v>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Quinta</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>Novembro Azul e movimento</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>ID 24</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>Bioimpedância: o que ela mostra</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>Pessoas, método, bastidores e prova</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J9" s="22" t="inlineStr">
+        <is>
+          <t>A balança não conta a história toda.</t>
+        </is>
+      </c>
+      <c r="K9" s="22" t="n"/>
+      <c r="L9" s="22" t="n"/>
+      <c r="M9" s="22" t="inlineStr">
+        <is>
+          <t>Siga para ver como cuidamos</t>
+        </is>
+      </c>
+      <c r="N9" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O9" s="22" t="inlineStr">
+        <is>
+          <t>Profissional do time + aparelho no espaço (sem colaborador atendido)</t>
+        </is>
+      </c>
+      <c r="P9" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q9" s="22" t="inlineStr">
+        <is>
+          <t>Mostrar o aparelho e a leitura genérica. Nenhum dado real na tela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="92" customHeight="1">
+      <c r="A10" s="21" t="n">
+        <v>46332</v>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>Sexta</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Novembro Azul e movimento</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>NOVO (no lugar do ID 25)</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Novembro Azul na empresa: o que vai além do laço azul</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>Saúde corporativa, NR-1 e B2B</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J10" s="22" t="inlineStr">
+        <is>
+          <t>Novembro Azul não cabe em um mês.</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="n"/>
+      <c r="L10" s="22" t="n"/>
+      <c r="M10" s="22" t="inlineStr">
+        <is>
+          <t>Mande para quem cuida das pessoas na sua empresa</t>
+        </is>
+      </c>
+      <c r="N10" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #novembroazul #saudedohomem #saudecorporativa #prevencao</t>
+        </is>
+      </c>
+      <c r="O10" s="22" t="inlineStr">
+        <is>
+          <t>Arte institucional (fairedu)</t>
+        </is>
+      </c>
+      <c r="P10" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q10" s="22" t="inlineStr">
+        <is>
+          <t>Mensagem para o RH: campanha de um mês não muda adesão; cuidado perto do time, o ano inteiro, sim. Gancho para o Escritório do Cuidado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="19" t="n">
+        <v>46333</v>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="20" t="n"/>
+      <c r="L11" s="20" t="n"/>
+      <c r="M11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q11" s="20" t="inlineStr">
+        <is>
+          <t>Fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="19" t="n">
+        <v>46334</v>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="20" t="n"/>
+      <c r="L12" s="20" t="n"/>
+      <c r="M12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q12" s="20" t="inlineStr">
+        <is>
+          <t>Fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="92" customHeight="1">
+      <c r="A13" s="21" t="n">
+        <v>46335</v>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>Sono e prova: Chemitec</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>ID 48 (antecipado de 09/12)</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>Adesão e retorno: Chemitec, 1º semestre de 2026</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>Autoridade, salvamento e compartilhamento</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>98% de adesão. Veja como.</t>
+        </is>
+      </c>
+      <c r="K13" s="22" t="n"/>
+      <c r="L13" s="22" t="n"/>
+      <c r="M13" s="22" t="inlineStr">
+        <is>
+          <t>Comente CUIDADO para saber como funcionaria na sua empresa</t>
+        </is>
+      </c>
+      <c r="N13" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #gestaodepessoas #absenteismo #rh</t>
+        </is>
+      </c>
+      <c r="O13" s="22" t="inlineStr">
+        <is>
+          <t>Arte institucional; logo círculo</t>
+        </is>
+      </c>
+      <c r="P13" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q13" s="22" t="inlineStr">
+        <is>
+          <t>Números liberados: 161 atendimentos, 48 colaboradores atendidos (98% de adesão), 81,3% voltaram para 2 ou mais atendimentos, 46 smartbands. Sempre agregado. Confirmar se a Chemitec topa coautoria (Collab). Stories: enquete "Como você dormiu esta semana?" (era o ID 26).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="92" customHeight="1">
+      <c r="A14" s="21" t="n">
+        <v>46336</v>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>Sono e prova: Chemitec</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>ID 27</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>Higiene do sono em 3 passos</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>Descoberta, educação e retenção</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>Três ajustes para dormir melhor hoje.</t>
+        </is>
+      </c>
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="22" t="inlineStr">
+        <is>
+          <t>Mande para quem vive cansado</t>
+        </is>
+      </c>
+      <c r="N14" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O14" s="22" t="inlineStr">
+        <is>
+          <t>Um profissional do time</t>
+        </is>
+      </c>
+      <c r="P14" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q14" s="22" t="inlineStr">
+        <is>
+          <t>Série 1 Minuto de Cuidado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="92" customHeight="1">
+      <c r="A15" s="21" t="n">
+        <v>46337</v>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Quarta</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Sono e prova: Chemitec</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>ID 28</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Pilar 3: Sono reparador</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>Autoridade, salvamento e compartilhamento</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Sono não é tempo perdido.</t>
+        </is>
+      </c>
+      <c r="K15" s="22" t="n"/>
+      <c r="L15" s="22" t="n"/>
+      <c r="M15" s="22" t="inlineStr">
+        <is>
+          <t>Salve este carrossel</t>
+        </is>
+      </c>
+      <c r="N15" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O15" s="22" t="inlineStr">
+        <is>
+          <t>Arte estilo pilares</t>
+        </is>
+      </c>
+      <c r="P15" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q15" s="22" t="inlineStr">
+        <is>
+          <t>Série 7 pilares.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="92" customHeight="1">
+      <c r="A16" s="21" t="n">
+        <v>46338</v>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>Quinta</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>Sono e prova: Chemitec</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>NOVO (no lugar do ID 29)</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>Adesão baixa não é culpa do colaborador</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>Pessoas, método, bastidores e prova</t>
+        </is>
+      </c>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I16" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Adesão baixa não é culpa do colaborador.</t>
+        </is>
+      </c>
+      <c r="K16" s="22" t="n"/>
+      <c r="L16" s="22" t="n"/>
+      <c r="M16" s="22" t="inlineStr">
+        <is>
+          <t>Comente CUIDADO</t>
+        </is>
+      </c>
+      <c r="N16" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #gestaodepessoas #absenteismo #rh</t>
+        </is>
+      </c>
+      <c r="O16" s="22" t="inlineStr">
+        <is>
+          <t>Narração + imagens do espaço; fecha com o depoimento A4 em card</t>
+        </is>
+      </c>
+      <c r="P16" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q16" s="22" t="inlineStr">
+        <is>
+          <t>Da estratégia (#15). Usa a Chemitec como prova e a posição 3 da voz: programa que ninguém usa é custo, não cuidado. O ID 29 (smartband e sono) vai para dezembro, junto do tema Tecnologia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="92" customHeight="1">
+      <c r="A17" s="21" t="n">
+        <v>46339</v>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>Sexta</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>Sono e prova: Chemitec</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>ID 30</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Sono, produtividade e segurança: atenção aos turnos na indústria</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>Saúde corporativa, NR-1 e B2B</t>
+        </is>
+      </c>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I17" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>Quem trabalha de noite dorme diferente.</t>
+        </is>
+      </c>
+      <c r="K17" s="22" t="n"/>
+      <c r="L17" s="22" t="n"/>
+      <c r="M17" s="22" t="inlineStr">
+        <is>
+          <t>Mande para o seu SESMT</t>
+        </is>
+      </c>
+      <c r="N17" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #nr1 #riscospsicossociais #gestaodepessoas</t>
+        </is>
+      </c>
+      <c r="O17" s="22" t="inlineStr">
+        <is>
+          <t>Arte institucional</t>
+        </is>
+      </c>
+      <c r="P17" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q17" s="22" t="inlineStr">
+        <is>
+          <t>Revisão técnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="19" t="n">
+        <v>46340</v>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Dia Mundial do Diabetes</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>Stories: Dia Mundial do Diabetes e Medicina do Estilo de Vida</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>Relacionamento</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>Stories</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · sequência de 3 a 5 telas com figurinha</t>
+        </is>
+      </c>
+      <c r="J18" s="20" t="inlineStr">
+        <is>
+          <t>Hoje é o Dia Mundial do Diabetes.</t>
+        </is>
+      </c>
+      <c r="K18" s="20" t="n"/>
+      <c r="L18" s="20" t="n"/>
+      <c r="M18" s="20" t="inlineStr">
+        <is>
+          <t>Figurinha de quiz sobre hábitos</t>
+        </is>
+      </c>
+      <c r="N18" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O18" s="20" t="inlineStr">
+        <is>
+          <t>Arte (logo coração)</t>
+        </is>
+      </c>
+      <c r="P18" s="20" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q18" s="20" t="inlineStr">
+        <is>
+          <t>Agendar na sexta. Educativo, sem promessa de resultado. Revisão técnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="19" t="n">
+        <v>46341</v>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+      <c r="M19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q19" s="20" t="inlineStr">
+        <is>
+          <t>Domingo (Proclamação da República).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="92" customHeight="1">
+      <c r="A20" s="21" t="n">
+        <v>46342</v>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>Saúde mental e NR-01</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>ID 33 (era 18/11)</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>Pilar 4: Saúde mental e estresse (com CVV 188)</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="inlineStr">
+        <is>
+          <t>Autoridade, salvamento e compartilhamento</t>
+        </is>
+      </c>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I20" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J20" s="22" t="inlineStr">
+        <is>
+          <t>Estresse não avisa quando passa do limite.</t>
+        </is>
+      </c>
+      <c r="K20" s="22" t="n"/>
+      <c r="L20" s="22" t="n"/>
+      <c r="M20" s="22" t="inlineStr">
+        <is>
+          <t>Salve e mande para alguém</t>
+        </is>
+      </c>
+      <c r="N20" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O20" s="22" t="inlineStr">
+        <is>
+          <t>Arte estilo pilares</t>
+        </is>
+      </c>
+      <c r="P20" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q20" s="22" t="inlineStr">
+        <is>
+          <t>Último slide com CVV 188. Stories: caixa "O que mais pesa na sua semana?" (era o ID 31).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="92" customHeight="1">
+      <c r="A21" s="21" t="n">
+        <v>46343</v>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Saúde mental e NR-01</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>ID 32</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>Respiração para momentos de tensão</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Descoberta, educação e retenção</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I21" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J21" s="22" t="inlineStr">
+        <is>
+          <t>Um minuto para baixar a tensão.</t>
+        </is>
+      </c>
+      <c r="K21" s="22" t="n"/>
+      <c r="L21" s="22" t="n"/>
+      <c r="M21" s="22" t="inlineStr">
+        <is>
+          <t>Salve para usar antes da próxima reunião</t>
+        </is>
+      </c>
+      <c r="N21" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O21" s="22" t="inlineStr">
+        <is>
+          <t>Profissional de psicologia para a câmera</t>
+        </is>
+      </c>
+      <c r="P21" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q21" s="22" t="inlineStr">
+        <is>
+          <t>Série 1 Minuto de Cuidado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="92" customHeight="1">
+      <c r="A22" s="21" t="n">
+        <v>46344</v>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Quarta</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Saúde mental e NR-01</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>ID 35 (era 20/11, feriado)</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>NR-01 e riscos psicossociais: o que muda para o RH + lançamento do guia</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>Saúde corporativa, NR-1 e B2B</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I22" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J22" s="22" t="inlineStr">
+        <is>
+          <t>NR-01 não é só uma planilha.</t>
+        </is>
+      </c>
+      <c r="K22" s="22" t="n"/>
+      <c r="L22" s="22" t="n"/>
+      <c r="M22" s="22" t="inlineStr">
+        <is>
+          <t>Comente CUIDADO e receba o guia de NR-01 para o RH</t>
+        </is>
+      </c>
+      <c r="N22" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #nr1 #riscospsicossociais #gestaodepessoas</t>
+        </is>
+      </c>
+      <c r="O22" s="22" t="inlineStr">
+        <is>
+          <t>Arte institucional; logo círculo</t>
+        </is>
+      </c>
+      <c r="P22" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q22" s="22" t="inlineStr">
+        <is>
+          <t>POST MAIS IMPORTANTE DO MÊS. Depende de: guia de NR-01 pronto e validado pelo Dr. Ronald, e resposta automática da palavra CUIDADO funcionando até 13/11. Fixar no perfil. Versão em PDF no LinkedIn no mesmo dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="92" customHeight="1">
+      <c r="A23" s="21" t="n">
+        <v>46345</v>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Quinta</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Saúde mental e NR-01</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>ID 34</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>Como funciona o atendimento psicológico: o que fica só entre você e o profissional</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>Pessoas, método, bastidores e prova</t>
+        </is>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I23" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J23" s="22" t="inlineStr">
+        <is>
+          <t>O que você conta fica aqui.</t>
+        </is>
+      </c>
+      <c r="K23" s="22" t="n"/>
+      <c r="L23" s="22" t="n"/>
+      <c r="M23" s="22" t="inlineStr">
+        <is>
+          <t>Siga para conhecer o Escritório do Cuidado</t>
+        </is>
+      </c>
+      <c r="N23" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O23" s="22" t="inlineStr">
+        <is>
+          <t>Profissional de psicologia para a câmera</t>
+        </is>
+      </c>
+      <c r="P23" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q23" s="22" t="inlineStr">
+        <is>
+          <t>Explicar que o RH só recebe indicadores do grupo, anonimizados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="19" t="n">
+        <v>46346</v>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Sexta</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>Feriado: Dia da Consciência Negra</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>Sem post no feed</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="20" t="n"/>
+      <c r="L24" s="20" t="n"/>
+      <c r="M24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q24" s="20" t="inlineStr">
+        <is>
+          <t>Feriado nacional, emenda com o fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="19" t="n">
+        <v>46347</v>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="20" t="n"/>
+      <c r="M25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q25" s="20" t="inlineStr">
+        <is>
+          <t>Fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="19" t="n">
+        <v>46348</v>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" s="20" t="n"/>
+      <c r="L26" s="20" t="n"/>
+      <c r="M26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q26" s="20" t="inlineStr">
+        <is>
+          <t>Fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="92" customHeight="1">
+      <c r="A27" s="21" t="n">
+        <v>46349</v>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Relações, propósito e conversão</t>
+        </is>
+      </c>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>ID 53 (antecipado de 16/12)</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="inlineStr">
+        <is>
+          <t>Case Hospital Dia Santo Amaro: de 34 para cerca de 20 reclamações por mês</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="inlineStr">
+        <is>
+          <t>Autoridade, salvamento e compartilhamento</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I27" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J27" s="22" t="inlineStr">
+        <is>
+          <t>De 34 para cerca de 20.</t>
+        </is>
+      </c>
+      <c r="K27" s="22" t="n"/>
+      <c r="L27" s="22" t="n"/>
+      <c r="M27" s="22" t="inlineStr">
+        <is>
+          <t>Comente CUIDADO</t>
+        </is>
+      </c>
+      <c r="N27" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #gestaodepessoas #absenteismo #rh</t>
+        </is>
+      </c>
+      <c r="O27" s="22" t="inlineStr">
+        <is>
+          <t>Arte institucional; logo círculo</t>
+        </is>
+      </c>
+      <c r="P27" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q27" s="22" t="inlineStr">
+        <is>
+          <t>Dados liberados: redução de cerca de 40%, conformidade média de 98,2%, apresentado em congresso internacional. Stories: "Quem faz diferença no seu dia de trabalho?" (era o ID 36).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="92" customHeight="1">
+      <c r="A28" s="21" t="n">
+        <v>46350</v>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>Relações, propósito e conversão</t>
+        </is>
+      </c>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>ID 37</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="inlineStr">
+        <is>
+          <t>Conexões no trabalho também são saúde</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="inlineStr">
+        <is>
+          <t>Descoberta, educação e retenção</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I28" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J28" s="22" t="inlineStr">
+        <is>
+          <t>Quem você procura num dia difícil?</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="n"/>
+      <c r="L28" s="22" t="n"/>
+      <c r="M28" s="22" t="inlineStr">
+        <is>
+          <t>Mande para essa pessoa</t>
+        </is>
+      </c>
+      <c r="N28" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O28" s="22" t="inlineStr">
+        <is>
+          <t>Dois integrantes do time em conversa</t>
+        </is>
+      </c>
+      <c r="P28" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q28" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="92" customHeight="1">
+      <c r="A29" s="21" t="n">
+        <v>46351</v>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>Quarta</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Relações, propósito e conversão</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>ID 38</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>Pilares 6 e 7: Relações sociais e Propósito</t>
+        </is>
+      </c>
+      <c r="G29" s="22" t="inlineStr">
+        <is>
+          <t>Autoridade, salvamento e compartilhamento</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I29" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J29" s="22" t="inlineStr">
+        <is>
+          <t>Relações e propósito também são saúde.</t>
+        </is>
+      </c>
+      <c r="K29" s="22" t="n"/>
+      <c r="L29" s="22" t="n"/>
+      <c r="M29" s="22" t="inlineStr">
+        <is>
+          <t>Salve este carrossel</t>
+        </is>
+      </c>
+      <c r="N29" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #medicinadoestilodevida #saudedotrabalhador #prevencao #saudecorporativa</t>
+        </is>
+      </c>
+      <c r="O29" s="22" t="inlineStr">
+        <is>
+          <t>Arte estilo pilares</t>
+        </is>
+      </c>
+      <c r="P29" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q29" s="22" t="inlineStr">
+        <is>
+          <t>Série 7 pilares.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="92" customHeight="1">
+      <c r="A30" s="21" t="n">
+        <v>46352</v>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>Quinta</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>Relações, propósito e conversão</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>ID 59 (antecipado de 17/12)</t>
+        </is>
+      </c>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>"Ela não gosta de gravar vídeo. Gravou um mesmo assim." (trechos em cards)</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>Pessoas, método, bastidores e prova</t>
+        </is>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="I30" s="22" t="inlineStr">
+        <is>
+          <t>9:16 · 1080x1920 · 30–45 s · texto na tela desde o 1º quadro</t>
+        </is>
+      </c>
+      <c r="J30" s="22" t="inlineStr">
+        <is>
+          <t>Ela não gosta de gravar vídeo.</t>
+        </is>
+      </c>
+      <c r="K30" s="22" t="n"/>
+      <c r="L30" s="22" t="n"/>
+      <c r="M30" s="22" t="inlineStr">
+        <is>
+          <t>Comente CUIDADO</t>
+        </is>
+      </c>
+      <c r="N30" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #gestaodepessoas #absenteismo #rh</t>
+        </is>
+      </c>
+      <c r="O30" s="22" t="inlineStr">
+        <is>
+          <t>Cards de texto com os trechos A6, A4 e A5 (logo coração)</t>
+        </is>
+      </c>
+      <c r="P30" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q30" s="22" t="inlineStr">
+        <is>
+          <t>O vídeo original NÃO é postado. Só trechos em texto, sem nome, rosto ou empresa (ver depoimentos.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="92" customHeight="1">
+      <c r="A31" s="21" t="n">
+        <v>46353</v>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>Sexta</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Relações, propósito e conversão</t>
+        </is>
+      </c>
+      <c r="E31" s="22" t="inlineStr">
+        <is>
+          <t>ID 63 + ID 65 (antecipados de dezembro)</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="inlineStr">
+        <is>
+          <t>Como começar: diagnóstico gratuito, proposta e implementação</t>
+        </is>
+      </c>
+      <c r="G31" s="22" t="inlineStr">
+        <is>
+          <t>Saúde corporativa, NR-1 e B2B</t>
+        </is>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I31" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J31" s="22" t="inlineStr">
+        <is>
+          <t>Como levar o cuidado para sua empresa.</t>
+        </is>
+      </c>
+      <c r="K31" s="22" t="n"/>
+      <c r="L31" s="22" t="n"/>
+      <c r="M31" s="22" t="inlineStr">
+        <is>
+          <t>Comente CUIDADO e agende o diagnóstico gratuito</t>
+        </is>
+      </c>
+      <c r="N31" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #nr1 #riscospsicossociais #gestaodepessoas</t>
+        </is>
+      </c>
+      <c r="O31" s="22" t="inlineStr">
+        <is>
+          <t>Arte institucional; logo círculo</t>
+        </is>
+      </c>
+      <c r="P31" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q31" s="22" t="inlineStr">
+        <is>
+          <t>Janela de orçamento 2027 do RH. É Black Friday: nada de linguagem de promoção ("só hoje", "aproveite"). Se preferir, trocar com o post de 26/11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="19" t="n">
+        <v>46354</v>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" s="20" t="n"/>
+      <c r="L32" s="20" t="n"/>
+      <c r="M32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q32" s="20" t="inlineStr">
+        <is>
+          <t>Fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="19" t="n">
+        <v>46355</v>
+      </c>
+      <c r="B33" s="20" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" s="20" t="n"/>
+      <c r="L33" s="20" t="n"/>
+      <c r="M33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P33" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q33" s="20" t="inlineStr">
+        <is>
+          <t>Fim de semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="92" customHeight="1">
+      <c r="A34" s="21" t="n">
+        <v>46356</v>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>Fechamento do mês</t>
+        </is>
+      </c>
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>ID 58 (antecipado de 16/12)</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>Depoimentos em texto: o cuidado na voz de quem é atendido</t>
+        </is>
+      </c>
+      <c r="G34" s="22" t="inlineStr">
+        <is>
+          <t>Marca, relacionamento e diferenciação</t>
+        </is>
+      </c>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="I34" s="22" t="inlineStr">
+        <is>
+          <t>4:5 · 1080x1350 · 8–10 slides · slide 2 entendível sozinho</t>
+        </is>
+      </c>
+      <c r="J34" s="22" t="inlineStr">
+        <is>
+          <t>O processo não precisa ser perfeito.</t>
+        </is>
+      </c>
+      <c r="K34" s="22" t="n"/>
+      <c r="L34" s="22" t="n"/>
+      <c r="M34" s="22" t="inlineStr">
+        <is>
+          <t>Comente CUIDADO</t>
+        </is>
+      </c>
+      <c r="N34" s="22" t="inlineStr">
+        <is>
+          <t>#fairhealth #saudecorporativa #gestaodepessoas #absenteismo #rh</t>
+        </is>
+      </c>
+      <c r="O34" s="22" t="inlineStr">
+        <is>
+          <t>Cards de texto (logo coração)</t>
+        </is>
+      </c>
+      <c r="P34" s="22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
+      <c r="Q34" s="22" t="inlineStr">
+        <is>
+          <t>Trechos B1, B2, B3, A1, A2 e A3 ("É mudança de cultura"). Assinatura: "Colaboradora atendida pelo Escritório do Cuidado". Fecha o mês de prova.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>Pendências para novembro funcionar</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="25" t="inlineStr">
+        <is>
+          <t>Até 30/10</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="F37" s="25" t="inlineStr">
+        <is>
+          <t>Roteiros dos Reels de 03 e 05/11 aprovados e gravados na diária de outubro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>Até 06/11</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="inlineStr">
+        <is>
+          <t>Dr. Ronald</t>
+        </is>
+      </c>
+      <c r="F38" s="25" t="inlineStr">
+        <is>
+          <t>Revisão técnica dos posts de Novembro Azul, sono, saúde mental e Dia do Diabetes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>Até 06/11</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr">
+        <is>
+          <t>Diretoria</t>
+        </is>
+      </c>
+      <c r="F39" s="25" t="inlineStr">
+        <is>
+          <t>Confirmar com Chemitec e Hospital Dia Santo Amaro o uso do nome e, se possível, post em coautoria (Collab).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>Até 13/11</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="inlineStr">
+        <is>
+          <t>Marketing + Dr. Ronald</t>
+        </is>
+      </c>
+      <c r="F40" s="25" t="inlineStr">
+        <is>
+          <t>Guia de NR-01 para o RH pronto e validado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>Até 13/11</t>
+        </is>
+      </c>
+      <c r="D41" s="25" t="inlineStr">
+        <is>
+          <t>Marketing + Comercial</t>
+        </is>
+      </c>
+      <c r="F41" s="25" t="inlineStr">
+        <is>
+          <t>Resposta automática da palavra CUIDADO no direct e página do diagnóstico gratuito no ar, com UTM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>Até 13/11</t>
+        </is>
+      </c>
+      <c r="D42" s="25" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="F42" s="25" t="inlineStr">
+        <is>
+          <t>Meta de diagnósticos de novembro e quem responde os leads em até 24 h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="24" t="inlineStr">
+        <is>
+          <t>O que saiu de novembro (vai para dezembro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="25" t="inlineStr">
+        <is>
+          <t>IDs 21, 26, 31, 36</t>
+        </is>
+      </c>
+      <c r="D45" s="25" t="inlineStr">
+        <is>
+          <t>Stories</t>
+        </is>
+      </c>
+      <c r="F45" s="25" t="inlineStr">
+        <is>
+          <t>Enquetes e caixas de pergunta viraram Stories nos mesmos temas (o formato nativo delas). As respostas podem virar carrossel em dezembro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>ID 22</t>
+        </is>
+      </c>
+      <c r="D46" s="25" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="F46" s="25" t="inlineStr">
+        <is>
+          <t>Pausa ativa de 1 minuto na mesa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>ID 25</t>
+        </is>
+      </c>
+      <c r="D47" s="25" t="inlineStr">
+        <is>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="F47" s="25" t="inlineStr">
+        <is>
+          <t>Sedentarismo no trabalho: o que o RH pode estimular (substituído pelo Novembro Azul na empresa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>ID 29</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="F48" s="25" t="inlineStr">
+        <is>
+          <t>O que a smartband mostra sobre o sono (junta com o tema Tecnologia).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>IDs 39, 40</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="inlineStr">
+        <is>
+          <t>Reel / Carrossel</t>
+        </is>
+      </c>
+      <c r="F49" s="25" t="inlineStr">
+        <is>
+          <t>Um dia com o time; Pertencimento, clima e retenção.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>IDs 41 a 45</t>
+        </is>
+      </c>
+      <c r="D50" s="25" t="inlineStr">
+        <is>
+          <t>Semana Tecnologia</t>
+        </is>
+      </c>
+      <c r="F50" s="25" t="inlineStr">
+        <is>
+          <t>Começa em dezembro. O cronograma de 90 dias precisa ser refeito a partir de 01/12, porque os IDs 48, 53, 58, 59, 63 e 65 vieram para novembro.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:Q34"/>
+  <mergeCells count="25">
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="F42:Q42"/>
+    <mergeCell ref="F45:Q45"/>
+    <mergeCell ref="F41:Q41"/>
+    <mergeCell ref="F50:Q50"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="F47:Q47"/>
+    <mergeCell ref="F38:Q38"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="F46:Q46"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="F37:Q37"/>
+    <mergeCell ref="F39:Q39"/>
+    <mergeCell ref="F48:Q48"/>
+    <mergeCell ref="F49:Q49"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="F40:Q40"/>
+  </mergeCells>
+  <conditionalFormatting sqref="P5:P34">
+    <cfRule type="expression" priority="1" dxfId="4">
+      <formula>$P5="Publicado"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="5">
+      <formula>$P5="Aprovado"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="6">
+      <formula>$P5="Em revisão"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="7">
+      <formula>$P5="Em produção"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="P5:P34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Listas!$C$1:$C$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="H5:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Listas!$D$1:$D$4</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0096C3BA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Novembro 2026 · FAIR HEALTH · Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Tema do mês: da intenção à evidência. Posts no feed às 7:30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Terça</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Quarta</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Quinta</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Sexta</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>1
+STORIES
+Novembro Azul começa hoje</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>2
+Feriado: Finados</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>3
+REEL
+1 Minuto de Cuidado: por que o homem só vai ao médico quando dói</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>4
+CARROSSEL
+Pilar 2: Atividade física</t>
+        </is>
+      </c>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>5
+REEL
+Bioimpedância: o que ela mostra</t>
+        </is>
+      </c>
+      <c r="F5" s="31" t="inlineStr">
+        <is>
+          <t>6
+CARROSSEL
+Novembro Azul na empresa: o que vai além do laço azul</t>
+        </is>
+      </c>
+      <c r="G5" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>9
+CARROSSEL
+Adesão e retorno: Chemitec, 1º semestre de 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>10
+REEL
+Higiene do sono em 3 passos</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>11
+CARROSSEL
+Pilar 3: Sono reparador</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>12
+REEL
+Adesão baixa não é culpa do colaborador</t>
+        </is>
+      </c>
+      <c r="F6" s="31" t="inlineStr">
+        <is>
+          <t>13
+CARROSSEL
+Sono, produtividade e segurança: atenção aos turnos na indústria</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>14
+STORIES
+Dia Mundial do Diabetes e Medicina do Estilo de Vida</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>16
+CARROSSEL
+Pilar 4: Saúde mental e estresse (com CVV 188)</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>17
+REEL
+Respiração para momentos de tensão</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>18
+CARROSSEL
+NR-01 e riscos psicossociais: o que muda para o RH + lançamento do guia</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>19
+REEL
+Como funciona o atendimento psicológico: o que fica só entre você e o profissional</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>20
+Feriado: Dia da Consciência Negra</t>
+        </is>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>23
+CARROSSEL
+Case Hospital Dia Santo Amaro: de 34 para cerca de 20 reclamações por mês</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>24
+REEL
+Conexões no trabalho também são saúde</t>
+        </is>
+      </c>
+      <c r="D8" s="31" t="inlineStr">
+        <is>
+          <t>25
+CARROSSEL
+Pilares 6 e 7: Relações sociais e Propósito</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>26
+REEL
+"Ela não gosta de gravar vídeo. Gravou um mesmo assim." (trechos em cards)</t>
+        </is>
+      </c>
+      <c r="F8" s="31" t="inlineStr">
+        <is>
+          <t>27
+CARROSSEL
+Como começar: diagnóstico gratuito, proposta e implementação</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="110" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>30
+CARROSSEL
+Depoimentos em texto: o cuidado na voz de quem é atendido</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Legenda das cores: verde = Reel · cinza-claro = Carrossel · amarelo = Stories. Detalhes de cada post na aba Novembro.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>